<commit_message>
chore(data-release): publish site data 2026-09-09 07:14:42 UTC
</commit_message>
<xml_diff>
--- a/diseases/d001/2026-2029.xlsx
+++ b/diseases/d001/2026-2029.xlsx
@@ -26737,12 +26737,12 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H156" t="inlineStr">
@@ -26767,12 +26767,12 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="N156" t="n">
@@ -26815,40 +26815,185 @@
       </c>
       <c r="AV156" t="inlineStr">
         <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="AW156" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="AX156" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="AY156" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AZ156" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="BA156" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="BB156" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="BC156" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>plague</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>鼠疫</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
+        <v>0</v>
+      </c>
+      <c r="R157" t="n">
+        <v>0</v>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO157" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP157" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR157" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS157" t="inlineStr"/>
+      <c r="AT157" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU157" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV157" t="inlineStr">
+        <is>
           <t>kdca_open_api</t>
         </is>
       </c>
-      <c r="AW156" t="inlineStr">
+      <c r="AW157" t="inlineStr">
         <is>
           <t>Korea KDCA EID</t>
         </is>
       </c>
-      <c r="AX156" t="inlineStr">
+      <c r="AX157" t="inlineStr">
         <is>
           <t>https://www.data.go.kr/data/15139178/openapi.do</t>
         </is>
       </c>
-      <c r="AY156" t="inlineStr">
+      <c r="AY157" t="inlineStr">
         <is>
           <t>open_api_or_portal_download</t>
         </is>
       </c>
-      <c r="AZ156" t="inlineStr">
+      <c r="AZ157" t="inlineStr">
         <is>
           <t>kdca_open_api</t>
         </is>
       </c>
-      <c r="BA156" t="inlineStr">
+      <c r="BA157" t="inlineStr">
         <is>
           <t>Korea KDCA EID</t>
         </is>
       </c>
-      <c r="BB156" t="inlineStr">
+      <c r="BB157" t="inlineStr">
         <is>
           <t>https://www.data.go.kr/data/15139178/openapi.do</t>
         </is>
       </c>
-      <c r="BC156" t="inlineStr">
+      <c r="BC157" t="inlineStr">
         <is>
           <t>open_api_or_portal_download</t>
         </is>
@@ -26970,7 +27115,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10">
@@ -26980,7 +27125,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-09-16 04:19:59 UTC
</commit_message>
<xml_diff>
--- a/diseases/d001/2026-2029.xlsx
+++ b/diseases/d001/2026-2029.xlsx
@@ -27541,6 +27541,151 @@
         </is>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>plague</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>鼠疫</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>0</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0</v>
+      </c>
+      <c r="R161" t="n">
+        <v>0</v>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO161" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP161" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR161" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS161" t="inlineStr"/>
+      <c r="AT161" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU161" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV161" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="AW161" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="AX161" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="AY161" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AZ161" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="BA161" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="BB161" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="BC161" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -27574,7 +27719,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-06</t>
         </is>
       </c>
     </row>
@@ -27657,7 +27802,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10">
@@ -27667,7 +27812,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
chore(data-release): publish site data 2026-10-15 09:09:10 UTC
</commit_message>
<xml_diff>
--- a/diseases/d001/2026-2029.xlsx
+++ b/diseases/d001/2026-2029.xlsx
@@ -41187,6 +41187,151 @@
         </is>
       </c>
     </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>plague</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>鼠疫</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>0</v>
+      </c>
+      <c r="O231" t="n">
+        <v>0</v>
+      </c>
+      <c r="R231" t="n">
+        <v>0</v>
+      </c>
+      <c r="S231" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO231" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP231" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR231" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS231" t="inlineStr"/>
+      <c r="AT231" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU231" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV231" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="AW231" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="AX231" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="AY231" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AZ231" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="BA231" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="BB231" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="BC231" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -41220,7 +41365,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-01</t>
+          <t>2026-10-04</t>
         </is>
       </c>
     </row>
@@ -41303,7 +41448,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="10">
@@ -41313,7 +41458,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="11">

</xml_diff>